<commit_message>
Building book with new crew chapter and table updates
</commit_message>
<xml_diff>
--- a/Index_table.xlsx
+++ b/Index_table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samantha.l.werner\Desktop\Github\READ-SSB-SSB_METRICS_CATALOG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D63BF98-0DF6-4F06-B713-078786763445}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CE4B69D-8DE1-46A6-9972-9FD141A1C11A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="249" yWindow="754" windowWidth="16414" windowHeight="7286" xr2:uid="{00B459D0-0E6D-413C-B001-630CD9B1DBF5}"/>
+    <workbookView xWindow="746" yWindow="1234" windowWidth="15334" windowHeight="8169" xr2:uid="{00B459D0-0E6D-413C-B001-630CD9B1DBF5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -95,7 +95,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="67">
   <si>
     <t xml:space="preserve">Metric Category </t>
   </si>
@@ -215,13 +215,94 @@
   </si>
   <si>
     <t>Gear type-level</t>
+  </si>
+  <si>
+    <t>Education</t>
+  </si>
+  <si>
+    <t>Race</t>
+  </si>
+  <si>
+    <t>Hispanic</t>
+  </si>
+  <si>
+    <t>Income</t>
+  </si>
+  <si>
+    <t>Metric Title</t>
+  </si>
+  <si>
+    <t>Primary Port</t>
+  </si>
+  <si>
+    <t>Primary Fishery Category</t>
+  </si>
+  <si>
+    <t>Age Category</t>
+  </si>
+  <si>
+    <t>Health Insurance</t>
+  </si>
+  <si>
+    <t>Marital Status</t>
+  </si>
+  <si>
+    <t>Job Satisfaction</t>
+  </si>
+  <si>
+    <t>Years Fishing</t>
+  </si>
+  <si>
+    <t>Owner Operator</t>
+  </si>
+  <si>
+    <t>Position On Current Vessel</t>
+  </si>
+  <si>
+    <t>Advise Young</t>
+  </si>
+  <si>
+    <t>Fish Again If Life Lived Over</t>
+  </si>
+  <si>
+    <t>Fishing Is Just A Job</t>
+  </si>
+  <si>
+    <t>Considered Leaving Industry</t>
+  </si>
+  <si>
+    <t>Participated In Fisheries Management</t>
+  </si>
+  <si>
+    <t>Rules &amp; Regulations Change Quickly</t>
+  </si>
+  <si>
+    <t>Fines Are Fair</t>
+  </si>
+  <si>
+    <t>Regulations Too Restrictive</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crew Metrics </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crew Survey Visualization Tool </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crew Survey Participants </t>
+  </si>
+  <si>
+    <t xml:space="preserve">N/A </t>
+  </si>
+  <si>
+    <t>2012/13, 2018/19, 2023/24</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -255,6 +336,18 @@
       <name val="Tahoma"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -264,7 +357,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -333,11 +426,22 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -364,6 +468,19 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -680,7 +797,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83D40A82-FAB7-4053-BBD9-44EE0830FAC1}">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F39"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="20.3828125" customWidth="1"/>
@@ -1031,7 +1148,448 @@
         <v>35</v>
       </c>
     </row>
+    <row r="18" spans="1:6" ht="28.3" x14ac:dyDescent="0.4">
+      <c r="A18" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D18" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="E18" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="F18" s="10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="28.3" x14ac:dyDescent="0.4">
+      <c r="A19" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="E19" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="F19" s="10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="28.3" x14ac:dyDescent="0.4">
+      <c r="A20" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D20" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="E20" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="F20" s="10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="28.3" x14ac:dyDescent="0.4">
+      <c r="A21" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B21" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D21" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="E21" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="F21" s="10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="28.3" x14ac:dyDescent="0.4">
+      <c r="A22" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B22" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D22" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="E22" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="F22" s="10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="28.3" x14ac:dyDescent="0.4">
+      <c r="A23" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B23" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D23" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="E23" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="F23" s="10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="28.3" x14ac:dyDescent="0.4">
+      <c r="A24" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B24" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D24" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="E24" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="F24" s="10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="28.3" x14ac:dyDescent="0.4">
+      <c r="A25" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B25" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D25" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="E25" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="F25" s="10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="28.3" x14ac:dyDescent="0.4">
+      <c r="A26" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B26" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D26" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="E26" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="F26" s="10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="28.3" x14ac:dyDescent="0.4">
+      <c r="A27" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B27" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D27" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="E27" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="F27" s="10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="28.3" x14ac:dyDescent="0.4">
+      <c r="A28" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B28" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D28" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="E28" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="F28" s="10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="28.3" x14ac:dyDescent="0.4">
+      <c r="A29" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B29" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D29" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="E29" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="F29" s="10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="28.3" x14ac:dyDescent="0.4">
+      <c r="A30" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B30" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="C30" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D30" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="E30" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="F30" s="10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="28.3" x14ac:dyDescent="0.4">
+      <c r="A31" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B31" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="C31" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D31" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="E31" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="F31" s="10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="28.3" x14ac:dyDescent="0.4">
+      <c r="A32" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B32" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="C32" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D32" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="E32" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="F32" s="10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="28.3" x14ac:dyDescent="0.4">
+      <c r="A33" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B33" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="C33" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D33" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="E33" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="F33" s="10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="28.3" x14ac:dyDescent="0.4">
+      <c r="A34" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B34" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="C34" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D34" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="E34" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="F34" s="10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="28.3" x14ac:dyDescent="0.4">
+      <c r="A35" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B35" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="C35" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D35" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="E35" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="F35" s="10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="28.3" x14ac:dyDescent="0.4">
+      <c r="A36" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B36" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="C36" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D36" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="E36" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="F36" s="10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="28.3" x14ac:dyDescent="0.4">
+      <c r="A37" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B37" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="C37" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D37" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="E37" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="F37" s="10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="28.3" x14ac:dyDescent="0.4">
+      <c r="A38" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B38" t="s">
+        <v>60</v>
+      </c>
+      <c r="C38" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D38" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="E38" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="F38" s="10" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="28.3" x14ac:dyDescent="0.4">
+      <c r="A39" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="B39" t="s">
+        <v>61</v>
+      </c>
+      <c r="C39" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D39" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="E39" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="F39" s="10" t="s">
+        <v>66</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>

</xml_diff>

<commit_message>
updated IO finalized table
</commit_message>
<xml_diff>
--- a/Index_table.xlsx
+++ b/Index_table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samantha.l.werner\Desktop\Github\READ-SSB-SSB_METRICS_CATALOG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C3634AD-39A5-49D7-97D2-F6BD1B72FF19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2CB1B69-1232-446F-9F4C-AD406682426C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22340" yWindow="790" windowWidth="14090" windowHeight="10090" xr2:uid="{00B459D0-0E6D-413C-B001-630CD9B1DBF5}"/>
+    <workbookView xWindow="22540" yWindow="1240" windowWidth="15770" windowHeight="9780" xr2:uid="{00B459D0-0E6D-413C-B001-630CD9B1DBF5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,64 +38,6 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>Samantha.L.Werner</author>
-  </authors>
-  <commentList>
-    <comment ref="F16" authorId="0" shapeId="0" xr:uid="{D36589CA-2959-4AA5-85D4-6BAB13642969}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Samantha.L.Werner:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="A17" authorId="0" shapeId="0" xr:uid="{EC8A217A-345F-42A9-ABA5-7EBA2FE0D0EC}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t>Samantha.L.Werner:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <charset val="1"/>
-          </rPr>
-          <t xml:space="preserve">
-</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Samantha.L.Werner</author>
@@ -154,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="722" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="746" uniqueCount="110">
   <si>
     <t xml:space="preserve">Metric Category </t>
   </si>
@@ -465,7 +407,59 @@
     <t>Gini Coefficeint  (Vessel Revenue)</t>
   </si>
   <si>
-    <t>Inequality Measures.</t>
+    <t>Inequality Measures</t>
+  </si>
+  <si>
+    <t>Employment</t>
+  </si>
+  <si>
+    <t>Direct Impacts</t>
+  </si>
+  <si>
+    <t>Indirect Impacts</t>
+  </si>
+  <si>
+    <t>Inducted Impacts</t>
+  </si>
+  <si>
+    <t>Input-Output Measures</t>
+  </si>
+  <si>
+    <t>Fleet Level (Gear type and vessel length)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Summary Group(s) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">(how units are grouped for summary) </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Unit of Response </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">(trip, vessel, individual) </t>
+    </r>
+  </si>
+  <si>
+    <t>Northeast Input Output Model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">State, Region </t>
   </si>
 </sst>
 </file>
@@ -1030,20 +1024,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83D40A82-FAB7-4053-BBD9-44EE0830FAC1}">
-  <dimension ref="A1:G49"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83D40A82-FAB7-4053-BBD9-44EE0830FAC1}">
+  <dimension ref="A1:G53"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="20.3828125" customWidth="1"/>
     <col min="2" max="2" width="11.53515625" customWidth="1"/>
     <col min="3" max="3" width="17.69140625" customWidth="1"/>
-    <col min="4" max="4" width="17.765625" customWidth="1"/>
-    <col min="5" max="5" width="15.3828125" customWidth="1"/>
+    <col min="4" max="4" width="15.3828125" customWidth="1"/>
+    <col min="5" max="5" width="17.765625" customWidth="1"/>
     <col min="6" max="6" width="21.15234375" customWidth="1"/>
     <col min="7" max="7" width="17.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" ht="57" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1054,10 +1048,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>4</v>
+        <v>107</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>3</v>
+        <v>106</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>5</v>
@@ -1077,10 +1071,10 @@
         <v>6</v>
       </c>
       <c r="D2" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" s="8" t="s">
         <v>35</v>
-      </c>
-      <c r="E2" s="8" t="s">
-        <v>15</v>
       </c>
       <c r="F2" s="8" t="s">
         <v>34</v>
@@ -1100,10 +1094,10 @@
         <v>6</v>
       </c>
       <c r="D3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>36</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>15</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>7</v>
@@ -1123,10 +1117,10 @@
         <v>8</v>
       </c>
       <c r="D4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="4" t="s">
         <v>37</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>15</v>
       </c>
       <c r="F4" s="4">
         <v>2022</v>
@@ -1146,10 +1140,10 @@
         <v>9</v>
       </c>
       <c r="D5" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="4" t="s">
         <v>37</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>15</v>
       </c>
       <c r="F5" s="4">
         <v>2022</v>
@@ -1169,10 +1163,10 @@
         <v>6</v>
       </c>
       <c r="D6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" s="4" t="s">
         <v>36</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>15</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>7</v>
@@ -1181,7 +1175,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A7" s="7" t="s">
         <v>96</v>
       </c>
@@ -1192,10 +1186,10 @@
         <v>6</v>
       </c>
       <c r="D7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="4" t="s">
         <v>36</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>15</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>7</v>
@@ -1215,10 +1209,10 @@
         <v>88</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F8" s="9" t="s">
         <v>34</v>
@@ -1238,10 +1232,10 @@
         <v>88</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F9" s="9" t="s">
         <v>34</v>
@@ -1261,10 +1255,10 @@
         <v>88</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F10" s="9" t="s">
         <v>34</v>
@@ -1284,10 +1278,10 @@
         <v>88</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>34</v>
@@ -1307,10 +1301,10 @@
         <v>88</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F12" s="9" t="s">
         <v>34</v>
@@ -1330,10 +1324,10 @@
         <v>88</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>34</v>
@@ -1353,10 +1347,10 @@
         <v>6</v>
       </c>
       <c r="D14" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E14" s="4" t="s">
         <v>36</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>15</v>
       </c>
       <c r="F14" s="4" t="s">
         <v>7</v>
@@ -1365,185 +1359,185 @@
         <v>75</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="51.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="5" t="s">
+    <row r="15" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A15" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="F15" s="4">
+        <v>2024</v>
+      </c>
+      <c r="G15" s="9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A16" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="F16" s="4">
+        <v>2024</v>
+      </c>
+      <c r="G16" s="9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A17" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="F17" s="4">
+        <v>2024</v>
+      </c>
+      <c r="G17" s="9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A18" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="F18" s="4">
+        <v>2024</v>
+      </c>
+      <c r="G18" s="9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="51.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A19" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B19" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C19" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="D19" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E19" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="E15" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="F15" s="6" t="s">
+      <c r="F19" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="G15" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="28.3" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A16" s="5" t="s">
+      <c r="G19" s="9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="28.3" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A20" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B20" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="C20" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D20" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="E20" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="E16" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="F16" s="5">
+      <c r="F20" s="5">
         <v>2022</v>
       </c>
-      <c r="G16" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="9" t="s">
+      <c r="G20" s="9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A21" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B21" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C21" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="D17" s="9" t="s">
+      <c r="D21" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="E21" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="E17" s="9" t="s">
+      <c r="F21" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="G21" s="9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="55.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A22" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="D22" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="F17" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="G17" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="55.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A18" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B18" s="9" t="s">
-        <v>24</v>
-      </c>
-      <c r="C18" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="D18" s="4" t="s">
+      <c r="E22" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="E18" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="F18" s="9" t="s">
+      <c r="F22" s="9" t="s">
         <v>7</v>
-      </c>
-      <c r="G18" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A19" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="D19" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="E19" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="F19" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="G19" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A20" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F20" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="G20" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A21" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F21" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="G21" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A22" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D22" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="E22" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F22" s="4" t="s">
-        <v>34</v>
       </c>
       <c r="G22" s="9" t="s">
         <v>75</v>
@@ -1553,20 +1547,20 @@
       <c r="A23" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B23" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C23" s="4" t="s">
+      <c r="B23" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C23" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D23" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="E23" s="4" t="s">
+      <c r="D23" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="F23" s="4" t="s">
-        <v>7</v>
+      <c r="E23" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>34</v>
       </c>
       <c r="G23" s="9" t="s">
         <v>75</v>
@@ -1577,19 +1571,19 @@
         <v>21</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D24" s="9" t="s">
-        <v>35</v>
+      <c r="D24" s="4" t="s">
+        <v>15</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>34</v>
+        <v>7</v>
       </c>
       <c r="G24" s="9" t="s">
         <v>75</v>
@@ -1597,45 +1591,45 @@
     </row>
     <row r="25" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A25" s="7" t="s">
-        <v>60</v>
+        <v>21</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>43</v>
+        <v>26</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D25" s="9" t="s">
-        <v>63</v>
+        <v>6</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>15</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>62</v>
+        <v>36</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>64</v>
+        <v>7</v>
       </c>
       <c r="G25" s="9" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A26" s="7" t="s">
-        <v>60</v>
+        <v>21</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D26" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="E26" s="4" t="s">
-        <v>62</v>
+        <v>6</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E26" s="9" t="s">
+        <v>35</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>64</v>
+        <v>34</v>
       </c>
       <c r="G26" s="9" t="s">
         <v>75</v>
@@ -1643,22 +1637,22 @@
     </row>
     <row r="27" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A27" s="7" t="s">
-        <v>60</v>
+        <v>21</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>45</v>
+        <v>29</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D27" s="9" t="s">
-        <v>63</v>
+        <v>6</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>15</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>62</v>
+        <v>36</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>64</v>
+        <v>7</v>
       </c>
       <c r="G27" s="9" t="s">
         <v>75</v>
@@ -1666,22 +1660,22 @@
     </row>
     <row r="28" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A28" s="7" t="s">
-        <v>60</v>
+        <v>21</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D28" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="E28" s="4" t="s">
-        <v>62</v>
+        <v>6</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E28" s="9" t="s">
+        <v>35</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>64</v>
+        <v>34</v>
       </c>
       <c r="G28" s="9" t="s">
         <v>75</v>
@@ -1692,16 +1686,16 @@
         <v>60</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D29" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="E29" s="4" t="s">
-        <v>62</v>
+      <c r="D29" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E29" s="9" t="s">
+        <v>63</v>
       </c>
       <c r="F29" s="4" t="s">
         <v>64</v>
@@ -1710,21 +1704,21 @@
         <v>75</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A30" s="7" t="s">
         <v>60</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D30" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="E30" s="4" t="s">
-        <v>62</v>
+      <c r="D30" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E30" s="9" t="s">
+        <v>63</v>
       </c>
       <c r="F30" s="4" t="s">
         <v>64</v>
@@ -1738,16 +1732,16 @@
         <v>60</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D31" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="E31" s="4" t="s">
-        <v>62</v>
+      <c r="D31" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E31" s="9" t="s">
+        <v>63</v>
       </c>
       <c r="F31" s="4" t="s">
         <v>64</v>
@@ -1761,16 +1755,16 @@
         <v>60</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D32" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="E32" s="4" t="s">
-        <v>62</v>
+      <c r="D32" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E32" s="9" t="s">
+        <v>63</v>
       </c>
       <c r="F32" s="4" t="s">
         <v>64</v>
@@ -1784,16 +1778,16 @@
         <v>60</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="C33" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D33" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="E33" s="4" t="s">
-        <v>62</v>
+      <c r="D33" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E33" s="9" t="s">
+        <v>63</v>
       </c>
       <c r="F33" s="4" t="s">
         <v>64</v>
@@ -1807,16 +1801,16 @@
         <v>60</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="C34" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D34" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="E34" s="4" t="s">
-        <v>62</v>
+      <c r="D34" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E34" s="9" t="s">
+        <v>63</v>
       </c>
       <c r="F34" s="4" t="s">
         <v>64</v>
@@ -1830,16 +1824,16 @@
         <v>60</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="C35" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D35" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="E35" s="4" t="s">
-        <v>62</v>
+      <c r="D35" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E35" s="9" t="s">
+        <v>63</v>
       </c>
       <c r="F35" s="4" t="s">
         <v>64</v>
@@ -1853,16 +1847,16 @@
         <v>60</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C36" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D36" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="E36" s="4" t="s">
-        <v>62</v>
+      <c r="D36" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E36" s="9" t="s">
+        <v>63</v>
       </c>
       <c r="F36" s="4" t="s">
         <v>64</v>
@@ -1871,21 +1865,21 @@
         <v>75</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A37" s="7" t="s">
         <v>60</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C37" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D37" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="E37" s="4" t="s">
-        <v>62</v>
+      <c r="D37" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E37" s="9" t="s">
+        <v>63</v>
       </c>
       <c r="F37" s="4" t="s">
         <v>64</v>
@@ -1899,16 +1893,16 @@
         <v>60</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C38" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D38" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="E38" s="4" t="s">
-        <v>62</v>
+      <c r="D38" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E38" s="9" t="s">
+        <v>63</v>
       </c>
       <c r="F38" s="4" t="s">
         <v>64</v>
@@ -1917,21 +1911,21 @@
         <v>75</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A39" s="7" t="s">
         <v>60</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D39" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="E39" s="4" t="s">
-        <v>62</v>
+      <c r="D39" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E39" s="9" t="s">
+        <v>63</v>
       </c>
       <c r="F39" s="4" t="s">
         <v>64</v>
@@ -1945,16 +1939,16 @@
         <v>60</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D40" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="E40" s="4" t="s">
-        <v>62</v>
+      <c r="D40" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E40" s="9" t="s">
+        <v>63</v>
       </c>
       <c r="F40" s="4" t="s">
         <v>64</v>
@@ -1968,16 +1962,16 @@
         <v>60</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C41" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D41" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="E41" s="4" t="s">
-        <v>62</v>
+      <c r="D41" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E41" s="9" t="s">
+        <v>63</v>
       </c>
       <c r="F41" s="4" t="s">
         <v>64</v>
@@ -1986,21 +1980,21 @@
         <v>75</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="57" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A42" s="7" t="s">
         <v>60</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C42" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D42" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="E42" s="4" t="s">
-        <v>62</v>
+      <c r="D42" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E42" s="9" t="s">
+        <v>63</v>
       </c>
       <c r="F42" s="4" t="s">
         <v>64</v>
@@ -2009,21 +2003,21 @@
         <v>75</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="57" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A43" s="7" t="s">
         <v>60</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C43" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D43" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="E43" s="4" t="s">
-        <v>62</v>
+      <c r="D43" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E43" s="9" t="s">
+        <v>63</v>
       </c>
       <c r="F43" s="4" t="s">
         <v>64</v>
@@ -2037,16 +2031,16 @@
         <v>60</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C44" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="D44" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="E44" s="4" t="s">
-        <v>62</v>
+      <c r="D44" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E44" s="9" t="s">
+        <v>63</v>
       </c>
       <c r="F44" s="4" t="s">
         <v>64</v>
@@ -2060,113 +2054,205 @@
         <v>60</v>
       </c>
       <c r="B45" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E45" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G45" s="9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" ht="57" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A46" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E46" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="F46" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G46" s="9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" ht="57" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A47" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E47" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="F47" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G47" s="9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A48" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E48" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="F48" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G48" s="9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A49" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="B49" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="C45" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D45" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="E45" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="F45" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="G45" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A46" s="10" t="s">
+      <c r="C49" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E49" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="F49" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G49" s="9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A50" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="B46" s="11" t="s">
+      <c r="B50" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="C46" s="4" t="s">
+      <c r="C50" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="D46" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="E46" s="4" t="s">
+      <c r="D50" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="F46" s="9" t="s">
+      <c r="E50" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="F50" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="G46" s="12" t="s">
+      <c r="G50" s="12" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="47" spans="1:7" ht="57" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A47" s="10" t="s">
+    <row r="51" spans="1:7" ht="57" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A51" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="B47" s="9" t="s">
+      <c r="B51" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="C47" s="9" t="s">
+      <c r="C51" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="D47" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="E47" s="9" t="s">
+      <c r="D51" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="F47" s="9" t="s">
+      <c r="E51" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="F51" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="G47" s="9" t="s">
+      <c r="G51" s="9" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A48" s="10" t="s">
+    <row r="52" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A52" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="B48" s="9" t="s">
+      <c r="B52" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="C48" s="9" t="s">
+      <c r="C52" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="D48" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="E48" s="9" t="s">
+      <c r="D52" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="F48" s="9" t="s">
+      <c r="E52" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="F52" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="G48" s="9" t="s">
+      <c r="G52" s="9" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="49" spans="1:7" ht="28.3" x14ac:dyDescent="0.4">
-      <c r="A49" s="10" t="s">
+    <row r="53" spans="1:7" ht="28.3" x14ac:dyDescent="0.4">
+      <c r="A53" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="B49" s="9" t="s">
+      <c r="B53" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="C49" s="9" t="s">
+      <c r="C53" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="D49" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="E49" s="9" t="s">
+      <c r="D53" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="F49" s="9" t="s">
+      <c r="E53" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="F53" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="G49" s="9" t="s">
+      <c r="G53" s="9" t="s">
         <v>87</v>
       </c>
     </row>
@@ -2174,7 +2260,6 @@
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -2621,7 +2706,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:8" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A18" s="9" t="s">
         <v>19</v>
       </c>
@@ -2647,7 +2732,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:8" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A19" s="7" t="s">
         <v>21</v>
       </c>
@@ -2673,7 +2758,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:8" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A20" s="7" t="s">
         <v>21</v>
       </c>
@@ -2699,7 +2784,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:8" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A21" s="7" t="s">
         <v>21</v>
       </c>

</xml_diff>

<commit_message>
ports added to index table
</commit_message>
<xml_diff>
--- a/Index_table.xlsx
+++ b/Index_table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samantha.l.werner\Desktop\Github\READ-SSB-SSB_METRICS_CATALOG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2CB1B69-1232-446F-9F4C-AD406682426C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABCA3E37-4771-43F1-B38C-9C765F6396BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22540" yWindow="1240" windowWidth="15770" windowHeight="9780" xr2:uid="{00B459D0-0E6D-413C-B001-630CD9B1DBF5}"/>
+    <workbookView xWindow="22550" yWindow="140" windowWidth="13300" windowHeight="10470" xr2:uid="{00B459D0-0E6D-413C-B001-630CD9B1DBF5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -96,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="746" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="774" uniqueCount="118">
   <si>
     <t xml:space="preserve">Metric Category </t>
   </si>
@@ -460,6 +460,30 @@
   </si>
   <si>
     <t xml:space="preserve">State, Region </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Port Activity Indicators  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Port Overall Activity score </t>
+  </si>
+  <si>
+    <t>Port Transaction Activity scor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Port Volume Activity </t>
+  </si>
+  <si>
+    <t>Port Permit Activity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Port Commercial Fishing Activity Indicator </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Port-level </t>
+  </si>
+  <si>
+    <t>Vessel-level</t>
   </si>
 </sst>
 </file>
@@ -1025,7 +1049,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83D40A82-FAB7-4053-BBD9-44EE0830FAC1}">
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="20.3828125" customWidth="1"/>
@@ -1508,7 +1532,7 @@
         <v>17</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>15</v>
+        <v>117</v>
       </c>
       <c r="E21" s="9" t="s">
         <v>20</v>
@@ -1531,7 +1555,7 @@
         <v>6</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>15</v>
+        <v>117</v>
       </c>
       <c r="E22" s="4" t="s">
         <v>36</v>
@@ -1553,8 +1577,8 @@
       <c r="C23" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="D23" s="6" t="s">
-        <v>15</v>
+      <c r="D23" s="9" t="s">
+        <v>117</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>35</v>
@@ -1576,8 +1600,8 @@
       <c r="C24" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D24" s="4" t="s">
-        <v>15</v>
+      <c r="D24" s="9" t="s">
+        <v>117</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>36</v>
@@ -1599,8 +1623,8 @@
       <c r="C25" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D25" s="4" t="s">
-        <v>15</v>
+      <c r="D25" s="9" t="s">
+        <v>117</v>
       </c>
       <c r="E25" s="4" t="s">
         <v>36</v>
@@ -1622,8 +1646,8 @@
       <c r="C26" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D26" s="4" t="s">
-        <v>15</v>
+      <c r="D26" s="9" t="s">
+        <v>117</v>
       </c>
       <c r="E26" s="9" t="s">
         <v>35</v>
@@ -1645,8 +1669,8 @@
       <c r="C27" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D27" s="4" t="s">
-        <v>15</v>
+      <c r="D27" s="9" t="s">
+        <v>117</v>
       </c>
       <c r="E27" s="4" t="s">
         <v>36</v>
@@ -1658,7 +1682,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:7" ht="44.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A28" s="7" t="s">
         <v>21</v>
       </c>
@@ -1668,8 +1692,8 @@
       <c r="C28" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D28" s="4" t="s">
-        <v>15</v>
+      <c r="D28" s="9" t="s">
+        <v>117</v>
       </c>
       <c r="E28" s="9" t="s">
         <v>35</v>
@@ -1681,93 +1705,93 @@
         <v>75</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:7" ht="44.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A29" s="7" t="s">
-        <v>60</v>
+        <v>110</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>43</v>
+        <v>111</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D29" s="4" t="s">
-        <v>62</v>
+        <v>115</v>
+      </c>
+      <c r="D29" s="9" t="s">
+        <v>116</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>63</v>
+        <v>116</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>64</v>
+        <v>18</v>
       </c>
       <c r="G29" s="9" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:7" ht="44.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A30" s="7" t="s">
-        <v>60</v>
+        <v>110</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>44</v>
+        <v>112</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D30" s="4" t="s">
-        <v>62</v>
+        <v>115</v>
+      </c>
+      <c r="D30" s="9" t="s">
+        <v>116</v>
       </c>
       <c r="E30" s="9" t="s">
-        <v>63</v>
+        <v>116</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>64</v>
+        <v>18</v>
       </c>
       <c r="G30" s="9" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:7" ht="44.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A31" s="7" t="s">
-        <v>60</v>
+        <v>110</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>45</v>
+        <v>113</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D31" s="4" t="s">
-        <v>62</v>
+        <v>115</v>
+      </c>
+      <c r="D31" s="9" t="s">
+        <v>116</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>63</v>
+        <v>116</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>64</v>
+        <v>18</v>
       </c>
       <c r="G31" s="9" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A32" s="7" t="s">
-        <v>60</v>
+        <v>110</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>39</v>
+        <v>114</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D32" s="4" t="s">
-        <v>62</v>
+        <v>115</v>
+      </c>
+      <c r="D32" s="9" t="s">
+        <v>116</v>
       </c>
       <c r="E32" s="9" t="s">
-        <v>63</v>
+        <v>116</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>64</v>
+        <v>18</v>
       </c>
       <c r="G32" s="9" t="s">
         <v>75</v>
@@ -1778,7 +1802,7 @@
         <v>60</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C33" s="4" t="s">
         <v>61</v>
@@ -1796,12 +1820,12 @@
         <v>75</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A34" s="7" t="s">
         <v>60</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C34" s="4" t="s">
         <v>61</v>
@@ -1824,7 +1848,7 @@
         <v>60</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C35" s="4" t="s">
         <v>61</v>
@@ -1847,7 +1871,7 @@
         <v>60</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="C36" s="4" t="s">
         <v>61</v>
@@ -1870,7 +1894,7 @@
         <v>60</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="C37" s="4" t="s">
         <v>61</v>
@@ -1893,7 +1917,7 @@
         <v>60</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="C38" s="4" t="s">
         <v>61</v>
@@ -1916,7 +1940,7 @@
         <v>60</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="C39" s="4" t="s">
         <v>61</v>
@@ -1939,7 +1963,7 @@
         <v>60</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>61</v>
@@ -1957,12 +1981,12 @@
         <v>75</v>
       </c>
     </row>
-    <row r="41" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A41" s="7" t="s">
         <v>60</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C41" s="4" t="s">
         <v>61</v>
@@ -1985,7 +2009,7 @@
         <v>60</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C42" s="4" t="s">
         <v>61</v>
@@ -2003,12 +2027,12 @@
         <v>75</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A43" s="7" t="s">
         <v>60</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="C43" s="4" t="s">
         <v>61</v>
@@ -2031,7 +2055,7 @@
         <v>60</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="C44" s="4" t="s">
         <v>61</v>
@@ -2054,7 +2078,7 @@
         <v>60</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C45" s="4" t="s">
         <v>61</v>
@@ -2072,12 +2096,12 @@
         <v>75</v>
       </c>
     </row>
-    <row r="46" spans="1:7" ht="57" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A46" s="7" t="s">
         <v>60</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C46" s="4" t="s">
         <v>61</v>
@@ -2095,12 +2119,12 @@
         <v>75</v>
       </c>
     </row>
-    <row r="47" spans="1:7" ht="57" thickBot="1" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A47" s="7" t="s">
         <v>60</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C47" s="4" t="s">
         <v>61</v>
@@ -2123,7 +2147,7 @@
         <v>60</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C48" s="4" t="s">
         <v>61</v>
@@ -2146,113 +2170,205 @@
         <v>60</v>
       </c>
       <c r="B49" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E49" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="F49" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G49" s="9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" ht="57" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A50" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E50" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="F50" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G50" s="9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" ht="57" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A51" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E51" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="F51" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G51" s="9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A52" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E52" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="F52" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G52" s="9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A53" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="B53" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="C49" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="D49" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="E49" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="F49" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="G49" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A50" s="10" t="s">
+      <c r="C53" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="E53" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="F53" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="G53" s="9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" ht="28.75" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A54" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="B50" s="11" t="s">
+      <c r="B54" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="C50" s="4" t="s">
+      <c r="C54" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="D50" s="4" t="s">
+      <c r="D54" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="E50" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="F50" s="9" t="s">
+      <c r="E54" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="F54" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="G50" s="12" t="s">
+      <c r="G54" s="12" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="51" spans="1:7" ht="57" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A51" s="10" t="s">
+    <row r="55" spans="1:7" ht="57" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A55" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="B51" s="9" t="s">
+      <c r="B55" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="C51" s="9" t="s">
+      <c r="C55" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="D51" s="9" t="s">
+      <c r="D55" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="E51" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="F51" s="9" t="s">
+      <c r="E55" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="F55" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="G51" s="9" t="s">
+      <c r="G55" s="9" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="52" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A52" s="10" t="s">
+    <row r="56" spans="1:7" ht="42.9" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A56" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="B52" s="9" t="s">
+      <c r="B56" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="C52" s="9" t="s">
+      <c r="C56" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="D52" s="9" t="s">
+      <c r="D56" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="E52" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="F52" s="9" t="s">
+      <c r="E56" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="F56" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="G52" s="9" t="s">
+      <c r="G56" s="9" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="53" spans="1:7" ht="28.3" x14ac:dyDescent="0.4">
-      <c r="A53" s="10" t="s">
+    <row r="57" spans="1:7" ht="28.3" x14ac:dyDescent="0.4">
+      <c r="A57" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="B53" s="9" t="s">
+      <c r="B57" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="C53" s="9" t="s">
+      <c r="C57" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="D53" s="9" t="s">
+      <c r="D57" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="E53" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="F53" s="9" t="s">
+      <c r="E57" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="F57" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="G53" s="9" t="s">
+      <c r="G57" s="9" t="s">
         <v>87</v>
       </c>
     </row>

</xml_diff>